<commit_message>
Evolution sur les ML 6b9f4c2382ca641594c413d968b63b2a848b2385
</commit_message>
<xml_diff>
--- a/htr-ML-Sections/ig/StructureDefinition-fr-lm-corps-document.xlsx
+++ b/htr-ML-Sections/ig/StructureDefinition-fr-lm-corps-document.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1375" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1406" uniqueCount="204">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-07T13:30:39+00:00</t>
+    <t>2026-05-12T13:21:37+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -588,6 +588,16 @@
   </si>
   <si>
     <t>Section object catalog</t>
+  </si>
+  <si>
+    <t>fr-lm-corps-document.recommendation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-recommendation
+</t>
+  </si>
+  <si>
+    <t>Section Recommandation</t>
   </si>
   <si>
     <t>fr-lm-corps-document.medicationDispensations</t>
@@ -959,7 +969,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AJ43"/>
+  <dimension ref="A1:AJ44"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="45.33984375" customWidth="true" bestFit="true"/>
@@ -5309,6 +5319,106 @@
         <v>73</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="s" s="2">
+        <v>201</v>
+      </c>
+      <c r="B44" t="s" s="2">
+        <v>201</v>
+      </c>
+      <c r="C44" s="2"/>
+      <c r="D44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E44" s="2"/>
+      <c r="F44" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K44" t="s" s="2">
+        <v>202</v>
+      </c>
+      <c r="L44" t="s" s="2">
+        <v>203</v>
+      </c>
+      <c r="M44" t="s" s="2">
+        <v>203</v>
+      </c>
+      <c r="N44" s="2"/>
+      <c r="O44" s="2"/>
+      <c r="P44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q44" s="2"/>
+      <c r="R44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF44" t="s" s="2">
+        <v>201</v>
+      </c>
+      <c r="AG44" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ44" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>